<commit_message>
I added decenter plots
</commit_message>
<xml_diff>
--- a/combined_tiptilt_data.xlsx
+++ b/combined_tiptilt_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakesutton/Documents/CMR Lab/NASA/Model T Paper/Flasher_heat_plotPython/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A51BFBB3-5B3B-BC47-A2AC-FD69F580864A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDDDF33-9407-9D4B-B773-1D110B6BDC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40860" yWindow="-18600" windowWidth="20120" windowHeight="25620" xr2:uid="{3FE5A48C-52D2-4C42-88F6-E05F5010E018}"/>
+    <workbookView xWindow="40860" yWindow="-18600" windowWidth="35420" windowHeight="25620" activeTab="3" xr2:uid="{3FE5A48C-52D2-4C42-88F6-E05F5010E018}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="47">
   <si>
     <t>Local</t>
   </si>
@@ -199,81 +199,6 @@
   </si>
   <si>
     <t>Deployment Success 3 Frame Scan</t>
-  </si>
-  <si>
-    <t>G5Ap5</t>
-  </si>
-  <si>
-    <t>G5Ap4</t>
-  </si>
-  <si>
-    <t>G5Ap3</t>
-  </si>
-  <si>
-    <t>G5Ap2</t>
-  </si>
-  <si>
-    <t>G5Ap1</t>
-  </si>
-  <si>
-    <t>G4Ap5</t>
-  </si>
-  <si>
-    <t>G4Ap4</t>
-  </si>
-  <si>
-    <t>G4Ap3</t>
-  </si>
-  <si>
-    <t>G4Ap2</t>
-  </si>
-  <si>
-    <t>G4Ap1</t>
-  </si>
-  <si>
-    <t>G3Ap5</t>
-  </si>
-  <si>
-    <t>G3Ap4</t>
-  </si>
-  <si>
-    <t>G3Ap3</t>
-  </si>
-  <si>
-    <t>G3Ap2</t>
-  </si>
-  <si>
-    <t>G3Ap1</t>
-  </si>
-  <si>
-    <t>G2Ap5</t>
-  </si>
-  <si>
-    <t>G2Ap4</t>
-  </si>
-  <si>
-    <t>G2Ap3</t>
-  </si>
-  <si>
-    <t>G2Ap2</t>
-  </si>
-  <si>
-    <t>G2Ap1</t>
-  </si>
-  <si>
-    <t>G1Ap5</t>
-  </si>
-  <si>
-    <t>G1Ap4</t>
-  </si>
-  <si>
-    <t>G1Ap3</t>
-  </si>
-  <si>
-    <t>G1Ap2</t>
-  </si>
-  <si>
-    <t>G1Ap1</t>
   </si>
   <si>
     <t>Deployment Success 4 Frame Scan</t>
@@ -23466,8 +23391,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7466856" y="9525"/>
-          <a:ext cx="5140938" cy="4399440"/>
+          <a:off x="7484918" y="9525"/>
+          <a:ext cx="5179080" cy="4408572"/>
           <a:chOff x="5022680" y="1344217"/>
           <a:chExt cx="3686110" cy="3561643"/>
         </a:xfrm>
@@ -33033,27 +32958,27 @@
         <v>36</v>
       </c>
       <c r="C33" s="3">
-        <f>AVERAGE(C7:C31)</f>
+        <f t="shared" ref="C33:H33" si="0">AVERAGE(C7:C31)</f>
         <v>0.20627301911899351</v>
       </c>
       <c r="D33" s="3">
-        <f>AVERAGE(D7:D31)</f>
+        <f t="shared" si="0"/>
         <v>-0.19713062338419557</v>
       </c>
       <c r="E33" s="3">
-        <f>AVERAGE(E7:E31)</f>
+        <f t="shared" si="0"/>
         <v>-2.9000000000000269E-2</v>
       </c>
       <c r="F33" s="3">
-        <f>AVERAGE(F7:F31)</f>
+        <f t="shared" si="0"/>
         <v>7.9248000000000554E-2</v>
       </c>
       <c r="G33" s="3">
-        <f>AVERAGE(G7:G31)</f>
+        <f t="shared" si="0"/>
         <v>-8.1280000000012904E-3</v>
       </c>
       <c r="H33" s="3">
-        <f>AVERAGE(H7:H31)</f>
+        <f t="shared" si="0"/>
         <v>-0.82814160000000003</v>
       </c>
       <c r="I33" s="3" t="s">
@@ -33906,27 +33831,27 @@
         <v>36</v>
       </c>
       <c r="C33" s="3">
-        <f>AVERAGE(C7:C31)</f>
+        <f t="shared" ref="C33:H33" si="0">AVERAGE(C7:C31)</f>
         <v>0.39423810537177617</v>
       </c>
       <c r="D33" s="3">
-        <f>AVERAGE(D7:D31)</f>
+        <f t="shared" si="0"/>
         <v>-0.79311330525811607</v>
       </c>
       <c r="E33" s="3">
-        <f>AVERAGE(E7:E31)</f>
+        <f t="shared" si="0"/>
         <v>-6.071999999999967E-2</v>
       </c>
       <c r="F33" s="3">
-        <f>AVERAGE(F7:F31)</f>
+        <f t="shared" si="0"/>
         <v>3.5560000000000903E-2</v>
       </c>
       <c r="G33" s="3">
-        <f>AVERAGE(G7:G31)</f>
+        <f t="shared" si="0"/>
         <v>-0.16154399999999891</v>
       </c>
       <c r="H33" s="3">
-        <f>AVERAGE(H7:H31)</f>
+        <f t="shared" si="0"/>
         <v>-0.59588400000000008</v>
       </c>
       <c r="I33" s="3" t="s">
@@ -34023,7 +33948,7 @@
   <sheetData>
     <row r="2" spans="2:9" ht="20" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -34111,7 +34036,7 @@
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B7" s="2" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3">
         <v>-0.11459163542067097</v>
@@ -34137,7 +34062,7 @@
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B8" s="2" t="s">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="C8" s="3">
         <v>0.51566897730870676</v>
@@ -34163,7 +34088,7 @@
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B9" s="2" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="C9" s="3">
         <v>0.11459163542067097</v>
@@ -34189,7 +34114,7 @@
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B10" s="2" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="C10" s="3">
         <v>-5.729578906238611E-2</v>
@@ -34215,7 +34140,7 @@
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B11" s="2" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="C11" s="3">
         <v>-0.22918372921171254</v>
@@ -34241,7 +34166,7 @@
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B12" s="2" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="C12" s="3">
         <v>-0.91677159063474134</v>
@@ -34267,7 +34192,7 @@
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B13" s="2" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="C13" s="3">
         <v>-0.85946892483581838</v>
@@ -34293,7 +34218,7 @@
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B14" s="2" t="s">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="C14" s="3">
         <v>-0.40107373207252695</v>
@@ -34319,7 +34244,7 @@
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B15" s="2" t="s">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="C15" s="3">
         <v>-0.17188759637130041</v>
@@ -34345,7 +34270,7 @@
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B16" s="2" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="C16" s="3">
         <v>-0.34377673975997053</v>
@@ -34371,7 +34296,7 @@
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B17" s="2" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="C17" s="3">
         <v>5.729578906238611E-2</v>
@@ -34397,7 +34322,7 @@
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B18" s="2" t="s">
-        <v>59</v>
+        <v>18</v>
       </c>
       <c r="C18" s="3">
         <v>-0.97407517351896133</v>
@@ -34423,7 +34348,7 @@
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B19" s="2" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="C19" s="3">
         <v>-0.57296734485715439</v>
@@ -34449,7 +34374,7 @@
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B20" s="2" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="C20" s="3">
         <v>1.6618105918581287</v>
@@ -34475,7 +34400,7 @@
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B21" s="2" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="C21" s="3">
         <v>1.6618105918581287</v>
@@ -34501,7 +34426,7 @@
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B22" s="2" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="C22" s="3">
         <v>0.74486611507034006</v>
@@ -34527,7 +34452,7 @@
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B23" s="2" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="C23" s="3">
         <v>2.1777639512803701</v>
@@ -34553,7 +34478,7 @@
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B24" s="2" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="C24" s="3">
         <v>2.2924427759558896</v>
@@ -34579,7 +34504,7 @@
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B25" s="2" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="C25" s="3">
         <v>2.1204278407307431</v>
@@ -34605,7 +34530,7 @@
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B26" s="2" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="C26" s="3">
         <v>1.7764537710952661</v>
@@ -34631,7 +34556,7 @@
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B27" s="2" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C27" s="3">
         <v>5.729578906238611E-2</v>
@@ -34657,7 +34582,7 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B28" s="2" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="C28" s="3">
         <v>0.28648009124091034</v>
@@ -34683,7 +34608,7 @@
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B29" s="2" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="C29" s="3">
         <v>-0.74486611507034006</v>
@@ -34709,7 +34634,7 @@
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B30" s="2" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="C30" s="3">
         <v>-0.45837112548533043</v>
@@ -34735,7 +34660,7 @@
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.15">
       <c r="B31" s="2" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C31" s="3">
         <v>-0.22918372921171254</v>
@@ -34764,27 +34689,27 @@
         <v>36</v>
       </c>
       <c r="C33" s="3">
-        <f>AVERAGE(C7:C31)</f>
+        <f t="shared" ref="C33:H33" si="0">AVERAGE(C7:C31)</f>
         <v>0.29573578777725212</v>
       </c>
       <c r="D33" s="3">
-        <f>AVERAGE(D7:D31)</f>
+        <f t="shared" si="0"/>
         <v>-0.76115974613075554</v>
       </c>
       <c r="E33" s="3">
-        <f>AVERAGE(E7:E31)</f>
+        <f t="shared" si="0"/>
         <v>-4.4999999999999929E-2</v>
       </c>
       <c r="F33" s="3">
-        <f>AVERAGE(F7:F31)</f>
+        <f t="shared" si="0"/>
         <v>3.9624000000000249E-2</v>
       </c>
       <c r="G33" s="3">
-        <f>AVERAGE(G7:G31)</f>
+        <f t="shared" si="0"/>
         <v>-0.10769600000000193</v>
       </c>
       <c r="H33" s="3">
-        <f>AVERAGE(H7:H31)</f>
+        <f t="shared" si="0"/>
         <v>-1.4698472</v>
       </c>
       <c r="I33" s="3" t="s">

</xml_diff>

<commit_message>
about to make a new branch
</commit_message>
<xml_diff>
--- a/combined_tiptilt_data.xlsx
+++ b/combined_tiptilt_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jakesutton/Documents/CMR Lab/NASA/Model T Paper/Flasher_heat_plotPython/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDDDF33-9407-9D4B-B773-1D110B6BDC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1E7955-6976-D34C-9481-EF9E12303A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40860" yWindow="-18600" windowWidth="35420" windowHeight="25620" activeTab="3" xr2:uid="{3FE5A48C-52D2-4C42-88F6-E05F5010E018}"/>
+    <workbookView xWindow="30220" yWindow="-20460" windowWidth="20520" windowHeight="26720" activeTab="2" xr2:uid="{3FE5A48C-52D2-4C42-88F6-E05F5010E018}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment1" sheetId="1" r:id="rId1"/>
@@ -195,13 +195,13 @@
     <t>THE OTHER SHEEST ARE THE UPDAED VERSION</t>
   </si>
   <si>
-    <t xml:space="preserve">THE DE CETNER VALUES HERE ARE NOT GOOD </t>
-  </si>
-  <si>
     <t>Deployment Success 3 Frame Scan</t>
   </si>
   <si>
     <t>Deployment Success 4 Frame Scan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THE GLOBAL DE CETNER VALUES HERE ARE NOT GOOD </t>
   </si>
 </sst>
 </file>
@@ -400,8 +400,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7270750" y="110490"/>
-          <a:ext cx="5168945" cy="4371032"/>
+          <a:off x="7244292" y="110490"/>
+          <a:ext cx="5124103" cy="4304199"/>
           <a:chOff x="5022680" y="1344217"/>
           <a:chExt cx="3686110" cy="3561643"/>
         </a:xfrm>
@@ -23391,8 +23391,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7484918" y="9525"/>
-          <a:ext cx="5179080" cy="4408572"/>
+          <a:off x="7450550" y="9525"/>
+          <a:ext cx="5124166" cy="4415047"/>
           <a:chOff x="5022680" y="1344217"/>
           <a:chExt cx="3686110" cy="3561643"/>
         </a:xfrm>
@@ -33061,7 +33061,7 @@
     </row>
     <row r="42" spans="2:9" x14ac:dyDescent="0.15">
       <c r="E42" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -33090,7 +33090,7 @@
   <sheetData>
     <row r="2" spans="2:9" ht="20" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -33948,7 +33948,7 @@
   <sheetData>
     <row r="2" spans="2:9" ht="20" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>

</xml_diff>